<commit_message>
Add Email Intelligence feature (offline email-archive analysis)
New `email-intelligence` plugin (Insights) that turns a downloaded
.eml/.txt + attachments archive into an offline people-and-life
intelligence base. No cloud, no AI, no database.

- Ingest/parse (MimeKit + .txt), dedupe (Message-Id + content hash),
  thread keys, message classification.
- Contacts + identity merge, signature details, relationship metrics
  (strength, dormant), topics, tone (offline lexicon), co-occurrence
  graph, per-person timelines.
- Life-data extraction (purchases/subscriptions/travel/accounts) and a
  hash-deduped document library.
- Append vs Overwrite mode to consolidate multiple archives into one
  de-duplicated dataset.
- Outputs: self-contained HTML5 report (tabbed), CSV/JSON/vCard/GraphML.
- 147 unit tests; full requirements + traceability docs. No host change.

build.ps1 -All: VERDICT PASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements/DigitalSecretary-Requirements.xlsx
+++ b/docs/requirements/DigitalSecretary-Requirements.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3566,6 +3566,2338 @@
       <c r="K57" s="2" t="inlineStr">
         <is>
           <t>docs/requirements/features/google-drive-downloader.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>EI-A1</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Scan archive</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Discover .eml/.txt files</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Recursively find .eml and .txt files in the chosen archive folder.</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Files under the folder are found; .eml preferred over its .txt sibling.</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>EI-A2</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Parse .eml</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Parse MIME via MimeKit</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Parse .eml headers, body and attachments with MimeKit.</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>From/To/Cc/Subject/Date/Message-Id and body are extracted.</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>EI-A3</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Parse .txt</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Parse the readable .txt form</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Parse the .txt form written by the downloaders (header lines, separator, body).</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>From/To/Date/Subject and body are read from a .txt file.</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>EI-A4</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Decode &amp; clean</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Decode encodings; HTML to text</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Decode MIME/encodings and convert HTML bodies to clean text; no mojibake.</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>An HTML body renders as readable text; whitespace normalized.</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>EI-B1</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Dedupe by Message-Id</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Remove exact duplicates</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Remove exact duplicate messages by Message-Id.</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Two messages with the same Message-Id collapse to one.</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>EI-B2</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Dedupe by content</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Collapse cross-account copies</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Remove near-duplicates by a content hash when Message-Id is absent.</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Identical mail with no Message-Id collapses to one.</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>EI-B3</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Thread key</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Group into conversations</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Compute a thread key from references or normalized subject.</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Re:/Fwd: subjects map to the same thread key.</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>EI-B4</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Classify</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Personal/Newsletter/Txn/Notification</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Classify each message using local sender/subject heuristics.</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>noreply senders are bulk; receipts transactional; verify is notification.</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>EI-C1</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Extract participants</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Every address + name</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Extract every participant (address + display name) across From/To/Cc.</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>All participants are captured with their display names.</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>EI-C2</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Detect owner</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Identify the archive owner</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Detect the owner from the most frequent sender; override allowed.</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>The most frequent From address is treated as the owner.</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>EI-C3</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Identity resolution</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Merge a person's addresses</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Merge addresses that share a normalized full name into one person.</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Two addresses with the same full name become one person.</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>EI-C4</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Person record</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Canonical person model</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Build a Person with canonical name, addresses and name variants.</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Each person lists all of their addresses.</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>EI-C5</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Signature details</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Phones + links from signatures</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Extract phone numbers and web/social links from message bodies.</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>A signature's phone and URL are captured.</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>EI-C6</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Contact export</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>vCard + CSV export</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Export the contact list as vCard and CSV for re-import.</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>A valid .vcf and a CSV with all contacts are written.</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>EI-D1</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Relationship metrics</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Counts, first/last contact</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Compute per-person sent/received counts and first/last contact.</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Direction counts and dates match the messages.</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>EI-D2</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Strength score</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Volume+reciprocity+recency</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Compute a transparent relationship strength score (0-100).</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>More frequent, recent, two-way contacts score higher.</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>EI-D3</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Dormant flag</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Flag lapsed contacts</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Flag historically frequent contacts with no recent contact.</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>A long-silent frequent contact is flagged dormant.</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>EI-D4</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Co-occurrence edges</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Who appears together</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Build weighted co-occurrence edges between people on shared emails.</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>People on the same email are linked, weighted by frequency.</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>EI-D5</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Org from email domain</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Derive an organization name from a non-free-mail email domain.</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Company domains yield an org; free-mail yields none.</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>EI-E1</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Topics</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Keyword extraction</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Extract per-person and global topics by local word frequency.</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Frequent non-stopwords surface as topics.</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>EI-E2</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Tone &amp; sentiment</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Lexicon tone (no AI)</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Score relationship tone with a bundled offline lexicon; label Positive/Neutral/Negative.</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Warm messages score positive; complaints negative; heuristic labelled.</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>EI-F1</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Purchases / receipts</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Extract orders + amounts</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Detect purchase/receipt/order emails and capture amount + currency.</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>A receipt email yields a Purchase item with its amount.</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>EI-F2</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Detect recurring/renewals</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Detect subscription/renewal/recurring emails.</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>A renewal email is categorized as Subscription.</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>EI-F3</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Detect trips/bookings</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Detect flight/hotel/booking-confirmation emails.</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>A flight confirmation is categorized as Travel.</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>EI-F4</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Account inventory</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Services signed up for</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Detect welcome/verify/reset emails to inventory account sign-ups.</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>A welcome/verify email is categorized as Account.</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>EI-F7</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Document library</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Deduped attachment library</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Collect attachments into a hash-deduped, type-classified document library.</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Identical attachments are counted once; each is typed (PDF/Image/...).</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>EI-G1</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>People search</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Type-ahead search</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Search people by name or email in the report.</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Typing filters the people list live.</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>EI-G2</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Dossier</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Per-person detail card</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Show a dossier with details, metrics and topics for a person.</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Selecting a person shows their full dossier.</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>EI-G4</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Drill-through</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Open original message</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Link timeline entries to their source message file.</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Each timeline entry links to its .eml/.txt source.</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>EI-G6</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Relationship history timeline</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Build an ordered per-person interaction timeline.</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>A person's interactions appear in date order with direction.</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>EI-H1</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Tabular output</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Excel-ready CSV sheets</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Write contacts/relationships as CSV (opens in Excel).</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>A Contacts.csv with a header and one row per person is written.</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>EI-H2</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Portable formats</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>JSON/vCard/GraphML</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Write JSON, vCard and GraphML companion outputs.</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>report.json, Contacts.vcf and network.graphml are written.</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>EI-H5</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>No database</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Files only; offline</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Write all outputs as files under the output folder; no database.</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Output folder contains files only; no DB; no network used.</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>EI-I1</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Idempotent re-run</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Re-run without duplicating</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Re-running on the same archive does not double-count (dedupe).</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>A second run yields the same counts.</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>EI-I4</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Append / overwrite</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Consolidate archives or replace</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Append merges a new archive with the persisted prior messages and re-dedupes; overwrite uses the current input only.</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Append across two archives yields one deduped dataset; overwrite replaces.</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>EI-J1</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>Configuration</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Folders + owner option</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Configure input/output folders and an optional owner address.</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Chosen folders and owner are used by the run.</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>EI-J2</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Progress &amp; cancel UI</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Bar + log + cancel</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Run on a background worker with a progress bar, log and cancel.</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>The bar advances; Cancel stops cleanly.</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>EI-J3</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Settings storage</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Persist; no secrets</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Persist settings under the feature data folder; store no secrets.</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Settings file holds folders + owner only.</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>EI-J4</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Open report</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Open the HTML report</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Offer to open the generated HTML report after a run.</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Open report launches index.html in the browser.</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>EI-J5</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Phased progress</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Per-phase progress + detail</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Report progress per phase with percent and current detail.</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Each phase reports a percent and a detail line.</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>EI-K1</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>HTML report tabs</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Tabbed HTML5 report</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Generate a single HTML report with tabbed views.</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>index.html opens with Overview/People/Timeline/Graph/Topics tabs.</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>EI-K2</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Folder data store</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Data beside the report</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Store the report's data in a data/ folder beside index.html.</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>data/data.js holds the model the page reads.</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>EI-K3</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Offline report</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>No CDN; opens from file://</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>The report is fully offline; data loads via a script tag.</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Opening index.html from disk works with no network.</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>EI-K4</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Client-side nav</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Search + tabs, no reload</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Navigate and search client-side without reloading.</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>Switching tabs and searching update without a reload.</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email Intelligence: native multi-sheet Excel (.xlsx) output
Add XlsxWriter, a dependency-free OOXML (SpreadsheetML) writer over
ZipArchive, plus WorkbookExporter. A run now also produces
EmailIntelligence.xlsx with Contacts / Life Data / Documents sheets and
typed numeric cells (validated with openpyxl). Chosen over a NuGet
spreadsheet library to keep the plugin fully offline and portable.

Requirement EI-H7 + traceability registered. 153 unit tests; coverage ~92%.
build.ps1 -All: VERDICT PASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements/DigitalSecretary-Requirements.xlsx
+++ b/docs/requirements/DigitalSecretary-Requirements.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5321,7 +5321,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>EI-I1</t>
+          <t>EI-H7</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Idempotent re-run</t>
+          <t>Excel workbook</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -5351,18 +5351,18 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Re-run without duplicating</t>
+          <t>Native multi-sheet .xlsx</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Re-running on the same archive does not double-count (dedupe).</t>
+          <t>Write a single multi-sheet Excel workbook (Contacts/Life Data/Documents) with a built-in OOXML writer, no dependency.</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>A second run yields the same counts.</t>
+          <t>EmailIntelligence.xlsx opens in Excel with the three sheets and typed numbers.</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
@@ -5374,7 +5374,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>EI-I4</t>
+          <t>EI-I1</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -5389,12 +5389,12 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Append / overwrite</t>
+          <t>Idempotent re-run</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5404,18 +5404,18 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Consolidate archives or replace</t>
+          <t>Re-run without duplicating</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Append merges a new archive with the persisted prior messages and re-dedupes; overwrite uses the current input only.</t>
+          <t>Re-running on the same archive does not double-count (dedupe).</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
       <c r="J92" s="2" t="inlineStr">
         <is>
-          <t>Append across two archives yields one deduped dataset; overwrite replaces.</t>
+          <t>A second run yields the same counts.</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
@@ -5427,7 +5427,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>EI-J1</t>
+          <t>EI-I4</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -5442,12 +5442,12 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Configuration</t>
+          <t>Append / overwrite</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -5457,18 +5457,18 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Folders + owner option</t>
+          <t>Consolidate archives or replace</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Configure input/output folders and an optional owner address.</t>
+          <t>Append merges a new archive with the persisted prior messages and re-dedupes; overwrite uses the current input only.</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
       <c r="J93" s="2" t="inlineStr">
         <is>
-          <t>Chosen folders and owner are used by the run.</t>
+          <t>Append across two archives yields one deduped dataset; overwrite replaces.</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
@@ -5480,7 +5480,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>EI-J2</t>
+          <t>EI-J1</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Progress &amp; cancel UI</t>
+          <t>Configuration</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -5510,18 +5510,18 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Bar + log + cancel</t>
+          <t>Folders + owner option</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Run on a background worker with a progress bar, log and cancel.</t>
+          <t>Configure input/output folders and an optional owner address.</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>The bar advances; Cancel stops cleanly.</t>
+          <t>Chosen folders and owner are used by the run.</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -5533,7 +5533,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>EI-J3</t>
+          <t>EI-J2</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -5548,7 +5548,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Settings storage</t>
+          <t>Progress &amp; cancel UI</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -5563,18 +5563,18 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Persist; no secrets</t>
+          <t>Bar + log + cancel</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Persist settings under the feature data folder; store no secrets.</t>
+          <t>Run on a background worker with a progress bar, log and cancel.</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>Settings file holds folders + owner only.</t>
+          <t>The bar advances; Cancel stops cleanly.</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
@@ -5586,7 +5586,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>EI-J4</t>
+          <t>EI-J3</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5601,12 +5601,12 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Open report</t>
+          <t>Settings storage</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -5616,18 +5616,18 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Open the HTML report</t>
+          <t>Persist; no secrets</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Offer to open the generated HTML report after a run.</t>
+          <t>Persist settings under the feature data folder; store no secrets.</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>Open report launches index.html in the browser.</t>
+          <t>Settings file holds folders + owner only.</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>EI-J5</t>
+          <t>EI-J4</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5654,12 +5654,12 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Phased progress</t>
+          <t>Open report</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -5669,18 +5669,18 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Per-phase progress + detail</t>
+          <t>Open the HTML report</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Report progress per phase with percent and current detail.</t>
+          <t>Offer to open the generated HTML report after a run.</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>Each phase reports a percent and a detail line.</t>
+          <t>Open report launches index.html in the browser.</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -5692,7 +5692,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>EI-K1</t>
+          <t>EI-J5</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5707,12 +5707,12 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>HTML report tabs</t>
+          <t>Phased progress</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -5722,18 +5722,18 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Tabbed HTML5 report</t>
+          <t>Per-phase progress + detail</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Generate a single HTML report with tabbed views.</t>
+          <t>Report progress per phase with percent and current detail.</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>index.html opens with Overview/People/Timeline/Graph/Topics tabs.</t>
+          <t>Each phase reports a percent and a detail line.</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -5745,7 +5745,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>EI-K2</t>
+          <t>EI-K1</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5760,12 +5760,12 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Folder data store</t>
+          <t>HTML report tabs</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -5775,18 +5775,18 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Data beside the report</t>
+          <t>Tabbed HTML5 report</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Store the report's data in a data/ folder beside index.html.</t>
+          <t>Generate a single HTML report with tabbed views.</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
       <c r="J99" s="2" t="inlineStr">
         <is>
-          <t>data/data.js holds the model the page reads.</t>
+          <t>index.html opens with Overview/People/Timeline/Graph/Topics tabs.</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
@@ -5798,7 +5798,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>EI-K3</t>
+          <t>EI-K2</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -5813,12 +5813,12 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Offline report</t>
+          <t>Folder data store</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -5828,18 +5828,18 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>No CDN; opens from file://</t>
+          <t>Data beside the report</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>The report is fully offline; data loads via a script tag.</t>
+          <t>Store the report's data in a data/ folder beside index.html.</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>Opening index.html from disk works with no network.</t>
+          <t>data/data.js holds the model the page reads.</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr">
@@ -5851,7 +5851,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>EI-K4</t>
+          <t>EI-K3</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -5866,12 +5866,12 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Client-side nav</t>
+          <t>Offline report</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -5881,21 +5881,74 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Search + tabs, no reload</t>
+          <t>No CDN; opens from file://</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Navigate and search client-side without reloading.</t>
+          <t>The report is fully offline; data loads via a script tag.</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
       <c r="J101" s="2" t="inlineStr">
         <is>
+          <t>Opening index.html from disk works with no network.</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>docs/requirements/features/email-intelligence.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>EI-K4</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Email Intelligence</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Client-side nav</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Search + tabs, no reload</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Navigate and search client-side without reloading.</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
           <t>Switching tabs and searching update without a reload.</t>
         </is>
       </c>
-      <c r="K101" s="2" t="inlineStr">
+      <c r="K102" s="2" t="inlineStr">
         <is>
           <t>docs/requirements/features/email-intelligence.md</t>
         </is>

</xml_diff>